<commit_message>
feat: mejora flujos y confirmaciones del panel admin
</commit_message>
<xml_diff>
--- a/docs/qa/Casos de prueba - Zunino Remates Web.xlsx
+++ b/docs/qa/Casos de prueba - Zunino Remates Web.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía y resumen" sheetId="1" r:id="Rea2415a7671d4c2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceso y sesión" sheetId="2" r:id="R43ada13e76024990"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gestión de remates" sheetId="3" r:id="Ree4ba70c346c4762"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo y lotes" sheetId="4" r:id="R6901a2c98f534608"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web pública" sheetId="5" r:id="R80ef7cbcba1d4e87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido y contacto" sheetId="6" r:id="R15cbfb5cd369431d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile y accesibilidad" sheetId="7" r:id="Rd1acb7cf161b4485"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos de prueba" sheetId="8" r:id="R056cc639b907400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía y resumen" sheetId="1" r:id="Rb7448020320a4ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceso y sesión" sheetId="2" r:id="Re4e55b60a1cd47bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gestión de remates" sheetId="3" r:id="R47f58692ad794ee8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo y lotes" sheetId="4" r:id="R8c687f97fce14b67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web pública" sheetId="5" r:id="R37f18cfef2aa4a65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido y contacto" sheetId="6" r:id="R717e688697164c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile y accesibilidad" sheetId="7" r:id="R99ee9df976c84736"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos de prueba" sheetId="8" r:id="Rda806432eae44589"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3572,7 +3572,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7f2bced5dead40a9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf82d4c5b996f4439"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4028,7 +4028,7 @@
       </x:c>
       <x:c r="E10" s="25" t="n">
         <x:f>COUNTA('Acceso y sesión'!$A$2:$A$200)+COUNTA('Gestión de remates'!$A$2:$A$200)+COUNTA('Catálogo y lotes'!$A$2:$A$200)+COUNTA('Web pública'!$A$2:$A$200)+COUNTA('Contenido y contacto'!$A$2:$A$200)+COUNTA('Mobile y accesibilidad'!$A$2:$A$200)</x:f>
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F10" s="23" t="n"/>
       <x:c r="G10" s="23" t="n"/>
@@ -4053,7 +4053,7 @@
       </x:c>
       <x:c r="E11" s="25" t="n">
         <x:f>COUNTIF('Acceso y sesión'!$J$2:$J$200,"No ejecutado")+COUNTIF('Gestión de remates'!$J$2:$J$200,"No ejecutado")+COUNTIF('Catálogo y lotes'!$J$2:$J$200,"No ejecutado")+COUNTIF('Web pública'!$J$2:$J$200,"No ejecutado")+COUNTIF('Contenido y contacto'!$J$2:$J$200,"No ejecutado")+COUNTIF('Mobile y accesibilidad'!$J$2:$J$200,"No ejecutado")</x:f>
-        <x:v>51</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F11" s="23" t="n"/>
       <x:c r="G11" s="23" t="n"/>
@@ -4078,7 +4078,7 @@
       </x:c>
       <x:c r="E12" s="25" t="n">
         <x:f>COUNTIF('Acceso y sesión'!$J$2:$J$200,"Aprobado")+COUNTIF('Gestión de remates'!$J$2:$J$200,"Aprobado")+COUNTIF('Catálogo y lotes'!$J$2:$J$200,"Aprobado")+COUNTIF('Web pública'!$J$2:$J$200,"Aprobado")+COUNTIF('Contenido y contacto'!$J$2:$J$200,"Aprobado")+COUNTIF('Mobile y accesibilidad'!$J$2:$J$200,"Aprobado")</x:f>
-        <x:v>28</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="F12" s="23" t="n"/>
       <x:c r="G12" s="23" t="n"/>
@@ -4180,7 +4180,7 @@
       </x:c>
       <x:c r="E17" s="25" t="n">
         <x:f>COUNTIF('Acceso y sesión'!$J$2:$J$200,"No ejecutado")+COUNTIF('Gestión de remates'!$J$2:$J$200,"No ejecutado")+COUNTIF('Catálogo y lotes'!$J$2:$J$200,"No ejecutado")+COUNTIF('Web pública'!$J$2:$J$200,"No ejecutado")+COUNTIF('Contenido y contacto'!$J$2:$J$200,"No ejecutado")+COUNTIF('Mobile y accesibilidad'!$J$2:$J$200,"No ejecutado")</x:f>
-        <x:v>51</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F17" s="23" t="n"/>
       <x:c r="G17" s="23" t="n"/>
@@ -4204,7 +4204,7 @@
       </x:c>
       <x:c r="E18" s="25" t="n">
         <x:f>COUNTIF('Acceso y sesión'!$J$2:$J$200,"Aprobado")+COUNTIF('Gestión de remates'!$J$2:$J$200,"Aprobado")+COUNTIF('Catálogo y lotes'!$J$2:$J$200,"Aprobado")+COUNTIF('Web pública'!$J$2:$J$200,"Aprobado")+COUNTIF('Contenido y contacto'!$J$2:$J$200,"Aprobado")+COUNTIF('Mobile y accesibilidad'!$J$2:$J$200,"Aprobado")</x:f>
-        <x:v>28</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="F18" s="23" t="n"/>
       <x:c r="G18" s="23" t="n"/>
@@ -4218,7 +4218,7 @@
       </x:c>
       <x:c r="B19" s="25" t="n">
         <x:f>COUNTA('Catálogo y lotes'!$A$2:$A$200)</x:f>
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C19" s="23" t="n"/>
       <x:c r="D19" s="25" t="inlineStr">
@@ -4307,7 +4307,7 @@
       </x:c>
       <x:c r="B23" s="26" t="n">
         <x:f>SUM(B17:B22)</x:f>
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C23" s="23" t="n"/>
       <x:c r="D23" s="23" t="n"/>
@@ -4355,7 +4355,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a52a7790f514eba"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7e4063530834238"/>
 </x:worksheet>
 </file>
 
@@ -4498,15 +4498,21 @@
           <x:t xml:space="preserve">Bloqueo de acceso válido o credenciales que no funcionan.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J2" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K2" s="36" t="n"/>
-      <x:c r="L2" s="36" t="n"/>
-      <x:c r="M2" s="37" t="n"/>
-      <x:c r="N2" s="38" t="n"/>
+      <x:c r="J2" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K2" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L2" s="36" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M2" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N2" s="38" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="96" customHeight="1">
       <x:c r="A3" s="12" t="inlineStr">
@@ -4556,15 +4562,21 @@
           <x:t xml:space="preserve">Acceso no autorizado.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J3" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K3" s="36" t="n"/>
-      <x:c r="L3" s="36" t="n"/>
-      <x:c r="M3" s="37" t="n"/>
-      <x:c r="N3" s="38" t="n"/>
+      <x:c r="J3" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K3" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L3" s="36" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M3" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N3" s="38" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="96" customHeight="1">
       <x:c r="A4" s="12" t="inlineStr">
@@ -4614,15 +4626,21 @@
           <x:t xml:space="preserve">Filtración de información de autenticación.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J4" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K4" s="36" t="n"/>
-      <x:c r="L4" s="36" t="n"/>
-      <x:c r="M4" s="37" t="n"/>
-      <x:c r="N4" s="38" t="n"/>
+      <x:c r="J4" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K4" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L4" s="36" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M4" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N4" s="38" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="96" customHeight="1">
       <x:c r="A5" s="12" t="inlineStr">
@@ -4672,15 +4690,21 @@
           <x:t xml:space="preserve">Ingreso accidental o mensaje confuso.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J5" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K5" s="36" t="n"/>
-      <x:c r="L5" s="36" t="n"/>
-      <x:c r="M5" s="37" t="n"/>
-      <x:c r="N5" s="38" t="n"/>
+      <x:c r="J5" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K5" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L5" s="36" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M5" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N5" s="38" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="96" customHeight="1">
       <x:c r="A6" s="12" t="inlineStr">
@@ -4729,15 +4753,21 @@
           <x:t xml:space="preserve">Pérdida inesperada de trabajo por recarga.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J6" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K6" s="36" t="n"/>
-      <x:c r="L6" s="36" t="n"/>
-      <x:c r="M6" s="37" t="n"/>
-      <x:c r="N6" s="38" t="n"/>
+      <x:c r="J6" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K6" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L6" s="36" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M6" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N6" s="38" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="96" customHeight="1">
       <x:c r="A7" s="12" t="inlineStr">
@@ -4786,15 +4816,21 @@
           <x:t xml:space="preserve">Sesión administrativa expuesta.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J7" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K7" s="36" t="n"/>
-      <x:c r="L7" s="36" t="n"/>
-      <x:c r="M7" s="37" t="n"/>
-      <x:c r="N7" s="38" t="n"/>
+      <x:c r="J7" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K7" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L7" s="36" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M7" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N7" s="38" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="96" customHeight="1">
       <x:c r="A8" s="13" t="inlineStr">
@@ -4843,15 +4879,21 @@
           <x:t xml:space="preserve">Pérdida de cambios o navegación inesperada.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J8" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K8" s="7" t="n"/>
-      <x:c r="L8" s="7" t="n"/>
-      <x:c r="M8" s="8" t="n"/>
-      <x:c r="N8" s="9" t="n"/>
+      <x:c r="J8" s="7" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K8" s="7" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L8" s="7" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M8" s="8" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N8" s="9" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="27.600000381469727" customHeight="1">
       <x:c r="A9" s="33" t="inlineStr">
@@ -4900,15 +4942,21 @@
           <x:t xml:space="preserve">Aviso permanente que confunde intentos posteriores.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J9" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K9" s="36" t="n"/>
-      <x:c r="L9" s="36" t="n"/>
-      <x:c r="M9" s="37" t="n"/>
-      <x:c r="N9" s="38" t="n"/>
+      <x:c r="J9" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K9" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L9" s="36" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M9" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N9" s="38" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="27.600000381469727" customHeight="1">
       <x:c r="A10" s="33" t="inlineStr">
@@ -4957,15 +5005,21 @@
           <x:t xml:space="preserve">No distinguir un error nuevo del anterior.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J10" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K10" s="36" t="n"/>
-      <x:c r="L10" s="36" t="n"/>
-      <x:c r="M10" s="37" t="n"/>
-      <x:c r="N10" s="38" t="n"/>
+      <x:c r="J10" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K10" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L10" s="36" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M10" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N10" s="38" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="41.400001525878906" customHeight="1">
       <x:c r="A11" s="33" t="inlineStr">
@@ -5015,15 +5069,21 @@
           <x:t xml:space="preserve">Pérdida del control de visibilidad.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J11" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K11" s="36" t="n"/>
-      <x:c r="L11" s="36" t="n"/>
-      <x:c r="M11" s="37" t="n"/>
-      <x:c r="N11" s="38" t="n"/>
+      <x:c r="J11" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K11" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L11" s="36" t="str">
+        <x:v>Verificado manualmente por Pablo.</x:v>
+      </x:c>
+      <x:c r="M11" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N11" s="38" t="str">
+        <x:v>Pablo</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="J2:J11">
@@ -5042,7 +5102,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70703a73711f40df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radfc2d67e88144c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7110,7 +7170,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76946582567d4761"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1994a1aabcc4b03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7253,15 +7313,21 @@
           <x:t xml:space="preserve">Sección rota cuando el array está vacío.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J2" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K2" s="36" t="n"/>
-      <x:c r="L2" s="36" t="n"/>
-      <x:c r="M2" s="37" t="n"/>
-      <x:c r="N2" s="38" t="n"/>
+      <x:c r="J2" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K2" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L2" s="36" t="str">
+        <x:v>Remate publicado sin lotes; el detalle no mostró una sección ni controles vacíos.</x:v>
+      </x:c>
+      <x:c r="M2" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N2" s="38" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="96" customHeight="1">
       <x:c r="A3" s="12" t="inlineStr">
@@ -7312,15 +7378,21 @@
           <x:t xml:space="preserve">Lote no persistido.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J3" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K3" s="36" t="n"/>
-      <x:c r="L3" s="36" t="n"/>
-      <x:c r="M3" s="37" t="n"/>
-      <x:c r="N3" s="38" t="n"/>
+      <x:c r="J3" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K3" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L3" s="36" t="str">
+        <x:v>Se cargaron seis PNG válidos y cada tarjeta mostró su nombre en el detalle público.</x:v>
+      </x:c>
+      <x:c r="M3" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N3" s="38" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="96" customHeight="1">
       <x:c r="A4" s="12" t="inlineStr">
@@ -7369,15 +7441,21 @@
           <x:t xml:space="preserve">Regresión conocida de animación y orden.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J4" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K4" s="36" t="n"/>
-      <x:c r="L4" s="36" t="n"/>
-      <x:c r="M4" s="37" t="n"/>
-      <x:c r="N4" s="38" t="n"/>
+      <x:c r="J4" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K4" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L4" s="36" t="str">
+        <x:v>Con seis lotes, ocho avances y ocho retrocesos recorrieron el carrusel circularmente y volvieron al primer lote.</x:v>
+      </x:c>
+      <x:c r="M4" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N4" s="38" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="96" customHeight="1">
       <x:c r="A5" s="12" t="inlineStr">
@@ -7426,73 +7504,37 @@
           <x:t xml:space="preserve">Condición de carrera en animación.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J5" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K5" s="36" t="n"/>
-      <x:c r="L5" s="36" t="n"/>
-      <x:c r="M5" s="37" t="n"/>
-      <x:c r="N5" s="38" t="n"/>
+      <x:c r="J5" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K5" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L5" s="36" t="str">
+        <x:v>Diez clics rápidos dejaron tres tarjetas válidas y el control habilitado luego de estabilizarse.</x:v>
+      </x:c>
+      <x:c r="M5" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N5" s="38" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="96" customHeight="1">
-      <x:c r="A6" s="12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CAT-010</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Media</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Imagen</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Imagen de lote rota</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Editar un lote.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F6" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">URL: https://ejemplo.invalid/imagen-inexistente.jpg
-Alt: Tractor rojo de prueba.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G6" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1. Publicar.
-2. Abrir detalle.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H6" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">La página no se rompe y el texto alternativo identifica la imagen. Registrar la presentación visual.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I6" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Dependencia de imágenes externas.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J6" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K6" s="36" t="n"/>
-      <x:c r="L6" s="36" t="n"/>
-      <x:c r="M6" s="37" t="n"/>
-      <x:c r="N6" s="38" t="n"/>
+      <x:c r="A6" s="12"/>
+      <x:c r="B6" s="10"/>
+      <x:c r="C6" s="36"/>
+      <x:c r="D6" s="36"/>
+      <x:c r="E6" s="36"/>
+      <x:c r="F6" s="36"/>
+      <x:c r="G6" s="36"/>
+      <x:c r="H6" s="36"/>
+      <x:c r="I6" s="36"/>
+      <x:c r="J6" s="36"/>
+      <x:c r="K6" s="36"/>
+      <x:c r="L6" s="36"/>
+      <x:c r="M6" s="37"/>
+      <x:c r="N6" s="38"/>
     </x:row>
     <x:row r="7" ht="96" customHeight="1">
       <x:c r="A7" s="12" t="inlineStr">
@@ -7541,15 +7583,21 @@
           <x:t xml:space="preserve">Saturación de almacenamiento local.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J7" s="36" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K7" s="36" t="n"/>
-      <x:c r="L7" s="36" t="n"/>
-      <x:c r="M7" s="37" t="n"/>
-      <x:c r="N7" s="38" t="n"/>
+      <x:c r="J7" s="36" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K7" s="36" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L7" s="36" t="str">
+        <x:v>El PNG de 700.001 bytes mostró el aviso de máximo excedido y no se agregó como lote.</x:v>
+      </x:c>
+      <x:c r="M7" s="37" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N7" s="38" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="96" customHeight="1">
       <x:c r="A8" s="13" t="inlineStr">
@@ -7599,15 +7647,21 @@
           <x:t xml:space="preserve">Modal atrapado o navegación inaccesible.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J8" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K8" s="7" t="n"/>
-      <x:c r="L8" s="7" t="n"/>
-      <x:c r="M8" s="8" t="n"/>
-      <x:c r="N8" s="9" t="n"/>
+      <x:c r="J8" s="7" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K8" s="7" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L8" s="7" t="str">
+        <x:v>El lightbox navegó entre lotes y cerró con X, Escape y clic fuera.</x:v>
+      </x:c>
+      <x:c r="M8" s="8" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N8" s="9" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="96" customHeight="1">
       <x:c r="A9" s="13" t="inlineStr">
@@ -7657,15 +7711,21 @@
           <x:t xml:space="preserve">Pérdida de archivos en una carga múltiple.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J9" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K9" s="7" t="n"/>
-      <x:c r="L9" s="7" t="n"/>
-      <x:c r="M9" s="8" t="n"/>
-      <x:c r="N9" s="9" t="n"/>
+      <x:c r="J9" s="7" t="str">
+        <x:v>No ejecutado</x:v>
+      </x:c>
+      <x:c r="K9" s="7" t="str">
+        <x:v>Pendiente de comprobación manual.</x:v>
+      </x:c>
+      <x:c r="L9" s="7" t="str">
+        <x:v>La automatización no puede arrastrar archivos desde el sistema operativo. La carga múltiple por selector se verificó en CAT-007.</x:v>
+      </x:c>
+      <x:c r="M9" s="8" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N9" s="9" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="96" customHeight="1">
       <x:c r="A10" s="13" t="inlineStr">
@@ -7715,15 +7775,21 @@
           <x:t xml:space="preserve">Imagen publicada sin identificación accesible.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J10" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K10" s="7" t="n"/>
-      <x:c r="L10" s="7" t="n"/>
-      <x:c r="M10" s="8" t="n"/>
-      <x:c r="N10" s="9" t="n"/>
+      <x:c r="J10" s="7" t="str">
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="K10" s="7" t="str">
+        <x:v>Coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L10" s="7" t="str">
+        <x:v>El guardado se bloqueó hasta completar el nombre de cada una de las seis imágenes.</x:v>
+      </x:c>
+      <x:c r="M10" s="8" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N10" s="9" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="96" customHeight="1">
       <x:c r="A11" s="13" t="inlineStr">
@@ -7775,15 +7841,21 @@
           <x:t xml:space="preserve">Obligatoriedad accidental de fotografías opcionales.</x:t>
         </x:is>
       </x:c>
-      <x:c r="J11" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No ejecutado</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K11" s="7" t="n"/>
-      <x:c r="L11" s="7" t="n"/>
-      <x:c r="M11" s="8" t="n"/>
-      <x:c r="N11" s="9" t="n"/>
+      <x:c r="J11" s="7" t="str">
+        <x:v>Fallido</x:v>
+      </x:c>
+      <x:c r="K11" s="7" t="str">
+        <x:v>No coincide con el resultado esperado.</x:v>
+      </x:c>
+      <x:c r="L11" s="7" t="str">
+        <x:v>No existe una acción para crear un lote sin fotografía: cada lote se genera únicamente al cargar una imagen.</x:v>
+      </x:c>
+      <x:c r="M11" s="8" t="str">
+        <x:v>01/09/2026</x:v>
+      </x:c>
+      <x:c r="N11" s="9" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="96" customHeight="1"/>
     <x:row r="13" ht="96" customHeight="1"/>
@@ -7804,7 +7876,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64068d3fea05479f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R130be1f22883434f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8545,7 +8617,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R502ec87b5d484260"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1aaca587cab64e2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9302,7 +9374,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf873aba85164cf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7d9d3d009546f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9964,7 +10036,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd88e504f932f400e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3f7c1aaad6c4071"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10485,7 +10557,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1dc5bd5ef5a4590"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R914b72c790094a5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>